<commit_message>
chunck fix and full context
</commit_message>
<xml_diff>
--- a/Bidder2offerevaluation/Bidder2offer_evaluation.xlsx
+++ b/Bidder2offerevaluation/Bidder2offer_evaluation.xlsx
@@ -576,7 +576,7 @@
       <c r="C4" s="6" t="inlineStr"/>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>Work order meeting experience criteria is not explicitly mentioned in the provided text.</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>The job involves designing, developing, and maintaining high-energy pulse arc (HEA) igniter systems for various fuels. The systems are designed to produce intense electrical sparks that ignite oil/gaseous particles, creating a flame pocket in the oil spray.</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -620,7 +620,7 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>The value of work or order required is not explicitly mentioned in the provided text.</t>
+          <t>174,930.00</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       <c r="C7" s="10" t="inlineStr"/>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>The value of work or order required is not explicitly mentioned in the provided text.</t>
+          <t>174,930.00</t>
         </is>
       </c>
     </row>
@@ -656,7 +656,7 @@
       <c r="C8" s="6" t="inlineStr"/>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>The value of work or order required is not explicitly mentioned in the provided text.</t>
+          <t>174,930.00</t>
         </is>
       </c>
     </row>
@@ -678,7 +678,7 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>The job involves designing, developing, and maintaining high-energy pulse arc (HEA) igniter systems for various fuels. The systems are designed to produce intense electrical sparks that ignite oil/gaseous particles, creating a flame pocket in the oil spray.</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
       <c r="C10" s="6" t="inlineStr"/>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Hindusthan Thermometers</t>
+          <t>Haldia Petrochemicals Limited</t>
         </is>
       </c>
     </row>
@@ -714,7 +714,7 @@
       <c r="C11" s="10" t="inlineStr"/>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>The details of the work order submitted include specifications for the HEA igniter system, such as the type of fuel it can ignite (high-speed diesel to heavy fuel oils and gases), the output voltage (2200V DC ± 10%), stored energy per spark (12 Joules), spark frequency (more than 4 sparks per second), and firing cycle (15 minutes on and 15 minutes off). The system should be designed for remote applications, such as igniting boilers and flare pilots.</t>
+          <t>Supply of Portable Ignitor and spares for Ignitors for unit-8 boiler</t>
         </is>
       </c>
     </row>
@@ -732,7 +732,7 @@
       <c r="C12" s="6" t="inlineStr"/>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>The value of work or order required is not explicitly mentioned in the provided text.</t>
+          <t>174,930.00</t>
         </is>
       </c>
     </row>
@@ -750,7 +750,7 @@
       <c r="C13" s="10" t="inlineStr"/>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>The value of work or order required is not explicitly mentioned in the provided text.</t>
+          <t>174,930.00</t>
         </is>
       </c>
     </row>
@@ -768,7 +768,7 @@
       <c r="C14" s="6" t="inlineStr"/>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>The value of work or order required is not explicitly mentioned in the provided text.</t>
+          <t>174,930.00</t>
         </is>
       </c>
     </row>
@@ -786,7 +786,7 @@
       <c r="C15" s="10" t="inlineStr"/>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>Subcontract approval submitted is not explicitly mentioned in the provided text.</t>
+          <t>Not Applicable</t>
         </is>
       </c>
     </row>
@@ -804,7 +804,7 @@
       <c r="C16" s="6" t="inlineStr"/>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>The value of work or order required is not explicitly mentioned in the provided text.</t>
+          <t>174,930.00</t>
         </is>
       </c>
     </row>
@@ -822,7 +822,7 @@
       <c r="C17" s="10" t="inlineStr"/>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>The value considered for technical evaluation is not explicitly mentioned in the provided text.</t>
+          <t>174,930.00</t>
         </is>
       </c>
     </row>
@@ -872,7 +872,7 @@
       <c r="C20" s="6" t="inlineStr"/>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>The value considered for technical evaluation is not explicitly mentioned in the provided text.</t>
+          <t>174,930.00</t>
         </is>
       </c>
     </row>
@@ -890,7 +890,7 @@
       <c r="C21" s="10" t="inlineStr"/>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>Reason for rejection is not explicitly mentioned in the provided text.</t>
+          <t>Not Applicable</t>
         </is>
       </c>
     </row>
@@ -914,7 +914,7 @@
       <c r="C23" s="10" t="inlineStr"/>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>The job involves designing, developing, and maintaining high-energy pulse arc (HEA) igniter systems for various fuels. The systems are designed to produce intense electrical sparks that ignite oil/gaseous particles, creating a flame pocket in the oil spray.</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -928,7 +928,7 @@
       <c r="C24" s="6" t="inlineStr"/>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>The value of work or order required is not explicitly mentioned in the provided text.</t>
+          <t>174,930.00</t>
         </is>
       </c>
     </row>
@@ -942,7 +942,7 @@
       <c r="C25" s="10" t="inlineStr"/>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>The details of the work order submitted include specifications for the HEA igniter system, such as the type of fuel it can ignite (high-speed diesel to heavy fuel oils and gases), the output voltage (2200V DC ± 10%), stored energy per spark (12 Joules), spark frequency (more than 4 sparks per second), and firing cycle (15 minutes on and 15 minutes off). The system should be designed for remote applications, such as igniting boilers and flare pilots.</t>
+          <t>Supply of Portable Ignitor and spares for Ignitors for unit-8 boiler</t>
         </is>
       </c>
     </row>
@@ -956,7 +956,7 @@
       <c r="C26" s="6" t="inlineStr"/>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>The work order number and date are not explicitly mentioned in the provided text.</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -970,7 +970,7 @@
       <c r="C27" s="10" t="inlineStr"/>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>The industry is related to industrial heating and combustion systems.</t>
+          <t>Petroleum / Petrochemical / Refinery / Power</t>
         </is>
       </c>
     </row>
@@ -984,7 +984,7 @@
       <c r="C28" s="6" t="inlineStr"/>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Hindusthan Thermometers</t>
+          <t>Haldia Petrochemicals Limited</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
       <c r="C29" s="10" t="inlineStr"/>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>Completion certificate details are not explicitly mentioned in the provided text.</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -1012,7 +1012,7 @@
       <c r="C30" s="6" t="inlineStr"/>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Executed value as per completion certificate is not explicitly mentioned in the provided text.</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -1026,7 +1026,7 @@
       <c r="C31" s="10" t="inlineStr"/>
       <c r="D31" s="11" t="inlineStr">
         <is>
-          <t>The value considered for technical evaluation is not explicitly mentioned in the provided text.</t>
+          <t>174,930.00</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1040,7 @@
       <c r="C32" s="6" t="inlineStr"/>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>Annualization of value is not explicitly mentioned in the provided text.</t>
+          <t>Not Applicable</t>
         </is>
       </c>
     </row>
@@ -1054,7 +1054,7 @@
       <c r="C33" s="10" t="inlineStr"/>
       <c r="D33" s="11" t="inlineStr">
         <is>
-          <t>Subcontract approval submitted is not explicitly mentioned in the provided text.</t>
+          <t>Not Applicable</t>
         </is>
       </c>
     </row>
@@ -1068,7 +1068,7 @@
       <c r="C34" s="6" t="inlineStr"/>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>Work order meeting experience criteria is not explicitly mentioned in the provided text.</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1082,7 @@
       <c r="C35" s="10" t="inlineStr"/>
       <c r="D35" s="11" t="inlineStr">
         <is>
-          <t>Additional technical PQC (Performance Quality Criteria) are not explicitly mentioned in the provided text.</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -1116,7 +1116,7 @@
       <c r="C38" s="6" t="inlineStr"/>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>Technical acceptance status is not explicitly mentioned in the provided text.</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -1130,7 +1130,7 @@
       <c r="C39" s="10" t="inlineStr"/>
       <c r="D39" s="11" t="inlineStr">
         <is>
-          <t>Reason for rejection is not explicitly mentioned in the provided text.</t>
+          <t>Not Applicable</t>
         </is>
       </c>
     </row>
@@ -1211,7 +1211,7 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>MSME</t>
+          <t>Not provided</t>
         </is>
       </c>
     </row>
@@ -1233,7 +1233,7 @@
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Not provided</t>
         </is>
       </c>
     </row>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not applicable</t>
         </is>
       </c>
     </row>
@@ -1299,7 +1299,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not applicable</t>
         </is>
       </c>
     </row>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Not applicable</t>
         </is>
       </c>
     </row>
@@ -1613,7 +1613,7 @@
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Not applicable</t>
         </is>
       </c>
     </row>
@@ -1635,7 +1635,7 @@
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Not applicable</t>
         </is>
       </c>
     </row>
@@ -1657,7 +1657,7 @@
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>MSME</t>
+          <t>Not provided</t>
         </is>
       </c>
     </row>
@@ -1679,7 +1679,7 @@
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Not applicable</t>
         </is>
       </c>
     </row>
@@ -1701,7 +1701,7 @@
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Not applicable</t>
         </is>
       </c>
     </row>
@@ -1723,7 +1723,7 @@
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Not applicable</t>
         </is>
       </c>
     </row>
@@ -1745,7 +1745,7 @@
       </c>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Not applicable</t>
         </is>
       </c>
     </row>
@@ -1767,7 +1767,7 @@
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Not applicable</t>
         </is>
       </c>
     </row>
@@ -1789,7 +1789,7 @@
       </c>
       <c r="D31" s="11" t="inlineStr">
         <is>
-          <t>Not provided</t>
+          <t>1126996</t>
         </is>
       </c>
     </row>
@@ -1811,7 +1811,7 @@
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Not applicable</t>
         </is>
       </c>
     </row>
@@ -1833,7 +1833,7 @@
       </c>
       <c r="D33" s="11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not applicable</t>
         </is>
       </c>
     </row>
@@ -2023,7 +2023,7 @@
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>Not Applicable</t>
+          <t>Not provided</t>
         </is>
       </c>
     </row>
@@ -2047,7 +2047,7 @@
       <c r="C44" s="6" t="inlineStr"/>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>MSME</t>
+          <t>Not provided</t>
         </is>
       </c>
     </row>
@@ -2061,7 +2061,7 @@
       <c r="C45" s="10" t="inlineStr"/>
       <c r="D45" s="11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Not provided</t>
         </is>
       </c>
     </row>
@@ -2089,7 +2089,7 @@
       <c r="C47" s="10" t="inlineStr"/>
       <c r="D47" s="11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not applicable</t>
         </is>
       </c>
     </row>
@@ -2103,7 +2103,7 @@
       <c r="C48" s="6" t="inlineStr"/>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not applicable</t>
         </is>
       </c>
     </row>
@@ -2243,7 +2243,7 @@
       <c r="C58" s="6" t="inlineStr"/>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>Not provided</t>
+          <t>1126996</t>
         </is>
       </c>
     </row>
@@ -2271,7 +2271,7 @@
       <c r="C60" s="6" t="inlineStr"/>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Not applicable</t>
         </is>
       </c>
     </row>
@@ -2285,7 +2285,7 @@
       <c r="C61" s="10" t="inlineStr"/>
       <c r="D61" s="11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not applicable</t>
         </is>
       </c>
     </row>
@@ -2299,7 +2299,7 @@
       <c r="C62" s="6" t="inlineStr"/>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not applicable</t>
         </is>
       </c>
     </row>
@@ -2313,7 +2313,7 @@
       <c r="C63" s="10" t="inlineStr"/>
       <c r="D63" s="11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not applicable</t>
         </is>
       </c>
     </row>
@@ -2327,7 +2327,7 @@
       <c r="C64" s="6" t="inlineStr"/>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not applicable</t>
         </is>
       </c>
     </row>
@@ -2341,7 +2341,7 @@
       <c r="C65" s="10" t="inlineStr"/>
       <c r="D65" s="11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not applicable</t>
         </is>
       </c>
     </row>
@@ -2355,7 +2355,7 @@
       <c r="C66" s="6" t="inlineStr"/>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not applicable</t>
         </is>
       </c>
     </row>
@@ -2369,7 +2369,7 @@
       <c r="C67" s="10" t="inlineStr"/>
       <c r="D67" s="11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not applicable</t>
         </is>
       </c>
     </row>
@@ -2383,7 +2383,7 @@
       <c r="C68" s="6" t="inlineStr"/>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not applicable</t>
         </is>
       </c>
     </row>
@@ -2397,7 +2397,7 @@
       <c r="C69" s="10" t="inlineStr"/>
       <c r="D69" s="11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not applicable</t>
         </is>
       </c>
     </row>
@@ -2411,7 +2411,7 @@
       <c r="C70" s="6" t="inlineStr"/>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not applicable</t>
         </is>
       </c>
     </row>
@@ -2425,7 +2425,7 @@
       <c r="C71" s="10" t="inlineStr"/>
       <c r="D71" s="11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not applicable</t>
         </is>
       </c>
     </row>
@@ -2505,7 +2505,7 @@
       <c r="C77" s="10" t="inlineStr"/>
       <c r="D77" s="11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not applicable</t>
         </is>
       </c>
     </row>
@@ -2543,7 +2543,7 @@
       <c r="C80" s="6" t="inlineStr"/>
       <c r="D80" s="7" t="inlineStr">
         <is>
-          <t>Not Applicable</t>
+          <t>Not provided</t>
         </is>
       </c>
     </row>
@@ -2634,7 +2634,7 @@
       <c r="C5" s="10" t="inlineStr"/>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Not Qualified</t>
         </is>
       </c>
     </row>
@@ -2656,7 +2656,7 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>High Energy Ignition Module</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -2678,7 +2678,7 @@
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>1234567890</t>
+          <t>3059539</t>
         </is>
       </c>
     </row>
@@ -2700,7 +2700,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>2023-12-31</t>
+          <t>January 30,2025</t>
         </is>
       </c>
     </row>
@@ -2722,7 +2722,7 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>1000.00</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -2744,7 +2744,7 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>John Doe</t>
+          <t>Haldia Petrochemicals Limited</t>
         </is>
       </c>
     </row>
@@ -2766,7 +2766,7 @@
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>John Doe</t>
+          <t>Haldia Petrochemicals Limited</t>
         </is>
       </c>
     </row>
@@ -2788,7 +2788,7 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>John Doe</t>
+          <t>Haldia Petrochemicals Limited</t>
         </is>
       </c>
     </row>
@@ -2810,7 +2810,7 @@
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>1000.00</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -2832,7 +2832,7 @@
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -2854,7 +2854,7 @@
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>950.00</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -2876,7 +2876,7 @@
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Not Applicable</t>
         </is>
       </c>
     </row>
@@ -2898,7 +2898,7 @@
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not Applicable</t>
         </is>
       </c>
     </row>
@@ -2922,7 +2922,7 @@
       <c r="C19" s="10" t="inlineStr"/>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>High Energy Ignition Module</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -2936,7 +2936,7 @@
       <c r="C20" s="6" t="inlineStr"/>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>1234567890</t>
+          <t>3059539</t>
         </is>
       </c>
     </row>
@@ -2950,7 +2950,7 @@
       <c r="C21" s="10" t="inlineStr"/>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>2023-12-31</t>
+          <t>January 30,2025</t>
         </is>
       </c>
     </row>
@@ -2964,7 +2964,7 @@
       <c r="C22" s="6" t="inlineStr"/>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>1000.00</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -2978,7 +2978,7 @@
       <c r="C23" s="10" t="inlineStr"/>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>John Doe</t>
+          <t>Haldia Petrochemicals Limited</t>
         </is>
       </c>
     </row>
@@ -2992,7 +2992,7 @@
       <c r="C24" s="6" t="inlineStr"/>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Jane Smith</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -3006,7 +3006,7 @@
       <c r="C25" s="10" t="inlineStr"/>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>Manufacturing</t>
+          <t>Petroleum/Petrochemical</t>
         </is>
       </c>
     </row>
@@ -3020,7 +3020,7 @@
       <c r="C26" s="6" t="inlineStr"/>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>950.00</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -3034,7 +3034,7 @@
       <c r="C27" s="10" t="inlineStr"/>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -3048,7 +3048,7 @@
       <c r="C28" s="6" t="inlineStr"/>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Applicable</t>
         </is>
       </c>
     </row>
@@ -3062,7 +3062,7 @@
       <c r="C29" s="10" t="inlineStr"/>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Not Applicable</t>
         </is>
       </c>
     </row>
@@ -3076,7 +3076,7 @@
       <c r="C30" s="6" t="inlineStr"/>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not Applicable</t>
         </is>
       </c>
     </row>
@@ -3100,7 +3100,7 @@
       <c r="C32" s="6" t="inlineStr"/>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Not Qualified</t>
         </is>
       </c>
     </row>
@@ -3114,7 +3114,7 @@
       <c r="C33" s="10" t="inlineStr"/>
       <c r="D33" s="11" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>The documents do not provide specific details about the bidder's past experience or project experience, which are required to meet the PQ Experience Criteria.</t>
         </is>
       </c>
     </row>
@@ -3209,7 +3209,7 @@
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>25%</t>
         </is>
       </c>
     </row>
@@ -3227,7 +3227,7 @@
       <c r="C6" s="6" t="inlineStr"/>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>50000000</t>
+          <t>38,24,620</t>
         </is>
       </c>
     </row>
@@ -3243,11 +3243,7 @@
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr"/>
-      <c r="D7" s="11" t="inlineStr">
-        <is>
-          <t>60000000</t>
-        </is>
-      </c>
+      <c r="D7" s="11" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -3261,11 +3257,7 @@
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr"/>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>70000000</t>
-        </is>
-      </c>
+      <c r="D8" s="7" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
@@ -3283,11 +3275,7 @@
           <t>Applicable / Not Applicable</t>
         </is>
       </c>
-      <c r="D9" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="D9" s="11" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr"/>
@@ -3309,7 +3297,7 @@
       <c r="C11" s="10" t="inlineStr"/>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>25%</t>
         </is>
       </c>
     </row>
@@ -3323,7 +3311,7 @@
       <c r="C12" s="6" t="inlineStr"/>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>50000000</t>
+          <t>38,24,620</t>
         </is>
       </c>
     </row>
@@ -3335,11 +3323,7 @@
         </is>
       </c>
       <c r="C13" s="10" t="inlineStr"/>
-      <c r="D13" s="11" t="inlineStr">
-        <is>
-          <t>60000000</t>
-        </is>
-      </c>
+      <c r="D13" s="11" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr"/>
@@ -3349,11 +3333,7 @@
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr"/>
-      <c r="D14" s="7" t="inlineStr">
-        <is>
-          <t>70000000</t>
-        </is>
-      </c>
+      <c r="D14" s="7" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr"/>
@@ -3363,11 +3343,7 @@
         </is>
       </c>
       <c r="C15" s="10" t="inlineStr"/>
-      <c r="D15" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="D15" s="11" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr"/>
@@ -3377,11 +3353,7 @@
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr"/>
-      <c r="D16" s="7" t="inlineStr">
-        <is>
-          <t>15000000</t>
-        </is>
-      </c>
+      <c r="D16" s="7" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr"/>
@@ -3403,7 +3375,7 @@
       <c r="C18" s="6" t="inlineStr"/>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Not applicable</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3468,7 @@
       <c r="C5" s="10" t="inlineStr"/>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -3510,7 +3482,7 @@
       <c r="C6" s="6" t="inlineStr"/>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>Yes - Signed &amp; Sealed</t>
         </is>
       </c>
     </row>
@@ -3524,7 +3496,7 @@
       <c r="C7" s="10" t="inlineStr"/>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -3536,11 +3508,7 @@
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr"/>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>The flame height is slightly higher than the specified range, but within acceptable limits.; The ignition delay time is longer than expected due to environmental factors.</t>
-        </is>
-      </c>
+      <c r="D8" s="7" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr"/>
@@ -3562,7 +3530,7 @@
       <c r="C10" s="6" t="inlineStr"/>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>Qualified</t>
         </is>
       </c>
     </row>
@@ -3576,7 +3544,7 @@
       <c r="C11" s="10" t="inlineStr"/>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>Not Applicable</t>
         </is>
       </c>
     </row>
@@ -3657,7 +3625,7 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>HT</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -3679,7 +3647,7 @@
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -3701,7 +3669,7 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -3745,7 +3713,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -3767,7 +3735,7 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>Details not provided in the text.</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -3789,7 +3757,7 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Details not provided in the text.</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -3811,7 +3779,7 @@
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -3833,7 +3801,7 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -3855,7 +3823,7 @@
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -3877,7 +3845,7 @@
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -3899,7 +3867,7 @@
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -3921,7 +3889,7 @@
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -3943,7 +3911,7 @@
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -3965,7 +3933,7 @@
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -3987,7 +3955,7 @@
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4009,7 +3977,7 @@
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4031,7 +3999,7 @@
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4053,7 +4021,7 @@
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4075,7 +4043,7 @@
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4097,7 +4065,7 @@
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4119,7 +4087,7 @@
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4141,7 +4109,7 @@
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4163,7 +4131,7 @@
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>Details not provided in the text.</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4185,7 +4153,7 @@
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4229,7 +4197,7 @@
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4219,7 @@
       </c>
       <c r="D31" s="11" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4273,7 +4241,7 @@
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>NIL</t>
         </is>
       </c>
     </row>
@@ -4297,7 +4265,7 @@
       <c r="C34" s="6" t="inlineStr"/>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>HT</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4311,7 +4279,7 @@
       <c r="C35" s="10" t="inlineStr"/>
       <c r="D35" s="11" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4325,7 +4293,7 @@
       <c r="C36" s="6" t="inlineStr"/>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4353,7 +4321,7 @@
       <c r="C38" s="6" t="inlineStr"/>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4367,7 +4335,7 @@
       <c r="C39" s="10" t="inlineStr"/>
       <c r="D39" s="11" t="inlineStr">
         <is>
-          <t>Details not provided in the text.</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4381,7 +4349,7 @@
       <c r="C40" s="6" t="inlineStr"/>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>Details not provided in the text.</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4395,7 +4363,7 @@
       <c r="C41" s="10" t="inlineStr"/>
       <c r="D41" s="11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4409,7 +4377,7 @@
       <c r="C42" s="6" t="inlineStr"/>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4423,7 +4391,7 @@
       <c r="C43" s="10" t="inlineStr"/>
       <c r="D43" s="11" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4437,7 +4405,7 @@
       <c r="C44" s="6" t="inlineStr"/>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4451,7 +4419,7 @@
       <c r="C45" s="10" t="inlineStr"/>
       <c r="D45" s="11" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4465,7 +4433,7 @@
       <c r="C46" s="6" t="inlineStr"/>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4479,7 +4447,7 @@
       <c r="C47" s="10" t="inlineStr"/>
       <c r="D47" s="11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4493,7 +4461,7 @@
       <c r="C48" s="6" t="inlineStr"/>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4507,7 +4475,7 @@
       <c r="C49" s="10" t="inlineStr"/>
       <c r="D49" s="11" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4521,7 +4489,7 @@
       <c r="C50" s="6" t="inlineStr"/>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4535,7 +4503,7 @@
       <c r="C51" s="10" t="inlineStr"/>
       <c r="D51" s="11" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4549,7 +4517,7 @@
       <c r="C52" s="6" t="inlineStr"/>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4563,7 +4531,7 @@
       <c r="C53" s="10" t="inlineStr"/>
       <c r="D53" s="11" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -4577,7 +4545,7 @@
       <c r="C54" s="6" t="inlineStr"/>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>NIL</t>
         </is>
       </c>
     </row>
@@ -4591,7 +4559,7 @@
       <c r="C55" s="10" t="inlineStr"/>
       <c r="D55" s="11" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -4605,7 +4573,7 @@
       <c r="C56" s="6" t="inlineStr"/>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4617,11 +4585,7 @@
         </is>
       </c>
       <c r="C57" s="10" t="inlineStr"/>
-      <c r="D57" s="11" t="inlineStr">
-        <is>
-          <t>Details not provided in the text.</t>
-        </is>
-      </c>
+      <c r="D57" s="11" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr"/>
@@ -4633,7 +4597,7 @@
       <c r="C58" s="6" t="inlineStr"/>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4647,7 +4611,7 @@
       <c r="C59" s="10" t="inlineStr"/>
       <c r="D59" s="11" t="inlineStr">
         <is>
-          <t>26/06/2020 to 25/06/2023</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4661,7 +4625,7 @@
       <c r="C60" s="6" t="inlineStr"/>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4675,7 +4639,7 @@
       <c r="C61" s="10" t="inlineStr"/>
       <c r="D61" s="11" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4677,7 @@
       <c r="C64" s="6" t="inlineStr"/>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>
@@ -4727,7 +4691,7 @@
       <c r="C65" s="10" t="inlineStr"/>
       <c r="D65" s="11" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not Found in Documents</t>
         </is>
       </c>
     </row>

</xml_diff>